<commit_message>
feat(backend): add JLPT & Kaiwa Google Sheet sync, formula decoder, and CVHT data scope
- Add staff_code to User, program_type/external_sync_key/program_metadata to Enrollment
- Add GoogleSheetSyncConfig and GoogleSheetRowState models + GOOGLE_SHEET_SYNC ImportType
- Implement sheet-sync.parser.ts (formula fallback decoding, JLPT Setting lookup, phone normalization, CareLog outcome classification)
- Implement sheet-sync.service.ts with SHA-256 file & row hash diffing and 5-minute background cron scheduler
- Add sheet-sync API endpoints and CVHT data scope filtering on /students, /enrollments, and /settings/users
- Update prisma/seed.ts and mock workbooks with CVHT01/02/03 assignments and integration tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data/cham_soc_hoc_vien_mock.xlsx
+++ b/docs/data/cham_soc_hoc_vien_mock.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="232">
   <si>
     <t>ff</t>
   </si>
@@ -77,7 +77,7 @@
     <t>Nghề nghiệp</t>
   </si>
   <si>
-    <t>Mô hình</t>
+    <t>CVHT</t>
   </si>
   <si>
     <t>Số buổi còn lại</t>
@@ -246,6 +246,9 @@
     <t>Kỹ sư phần mềm</t>
   </si>
   <si>
+    <t>CVHT01</t>
+  </si>
+  <si>
     <t>Đang học</t>
   </si>
   <si>
@@ -301,6 +304,9 @@
     <t>Nhân viên văn phòng</t>
   </si>
   <si>
+    <t>CVHT02</t>
+  </si>
+  <si>
     <t>canhnt/quyentn</t>
   </si>
   <si>
@@ -332,6 +338,9 @@
   </si>
   <si>
     <t>Quản lý dự án</t>
+  </si>
+  <si>
+    <t>CVHT03</t>
   </si>
   <si>
     <t>19h00</t>
@@ -679,6 +688,9 @@
   </si>
   <si>
     <t>Tháng 3</t>
+  </si>
+  <si>
+    <t>Mô hình</t>
   </si>
   <si>
     <t>Tổng số buổi đã học</t>
@@ -2156,7 +2168,7 @@
         <v>75</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="T4" s="37">
         <v>40</v>
@@ -2165,16 +2177,16 @@
         <v>46037</v>
       </c>
       <c r="V4" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W4" s="39">
         <v>46127</v>
       </c>
       <c r="X4" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Y4" s="33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Z4" s="33">
         <v>30</v>
@@ -2185,13 +2197,13 @@
       <c r="AD4" s="12"/>
       <c r="AE4" s="12"/>
       <c r="AF4" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AG4" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AH4" s="13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="AI4" s="40"/>
       <c r="AJ4" s="12"/>
@@ -2204,10 +2216,10 @@
       <c r="AM4" s="12"/>
       <c r="AN4" s="12"/>
       <c r="AO4" s="13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AP4" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AQ4" s="12"/>
       <c r="AR4" s="12"/>
@@ -2236,28 +2248,28 @@
     </row>
     <row r="5" ht="31.5" customHeight="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B5" s="34">
         <v>46034.38541666667</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>63</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G5" s="33" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I5" s="12" t="s">
         <v>68</v>
@@ -2266,13 +2278,13 @@
         <v>69</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L5" s="12" t="s">
         <v>71</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N5" s="35">
         <v>90</v>
@@ -2281,16 +2293,16 @@
         <v>73</v>
       </c>
       <c r="P5" s="12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q5" s="36">
         <v>36032</v>
       </c>
       <c r="R5" s="12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="S5" s="12" t="s">
-        <v>73</v>
+        <v>95</v>
       </c>
       <c r="T5" s="37">
         <v>75</v>
@@ -2299,16 +2311,16 @@
         <v>46040</v>
       </c>
       <c r="V5" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W5" s="38">
         <v>46191</v>
       </c>
       <c r="X5" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Y5" s="33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Z5" s="33">
         <v>30</v>
@@ -2319,30 +2331,30 @@
       <c r="AD5" s="12"/>
       <c r="AE5" s="12"/>
       <c r="AF5" s="12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AG5" s="12" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AH5" s="13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AI5" s="40"/>
       <c r="AJ5" s="33">
         <v>56</v>
       </c>
       <c r="AK5" s="41" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AL5" s="12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AM5" s="12"/>
       <c r="AN5" s="12"/>
       <c r="AO5" s="12"/>
       <c r="AP5" s="12"/>
       <c r="AQ5" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AR5" s="12"/>
       <c r="AS5" s="12"/>
@@ -2372,7 +2384,7 @@
     </row>
     <row r="6" ht="36.75" customHeight="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B6" s="34">
         <v>46036.69791666667</v>
@@ -2384,16 +2396,16 @@
         <v>63</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F6" s="12" t="s">
         <v>65</v>
       </c>
       <c r="G6" s="33" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I6" s="12" t="s">
         <v>68</v>
@@ -2402,13 +2414,13 @@
         <v>69</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="L6" s="12" t="s">
         <v>71</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N6" s="35">
         <v>60</v>
@@ -2417,16 +2429,16 @@
         <v>73</v>
       </c>
       <c r="P6" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="Q6" s="36">
         <v>34278</v>
       </c>
       <c r="R6" s="12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="S6" s="12" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="T6" s="37">
         <v>50</v>
@@ -2435,16 +2447,16 @@
         <v>46042</v>
       </c>
       <c r="V6" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W6" s="39">
         <v>46162</v>
       </c>
       <c r="X6" s="12" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="Y6" s="33" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="Z6" s="33">
         <v>30</v>
@@ -2455,29 +2467,29 @@
       <c r="AD6" s="12"/>
       <c r="AE6" s="12"/>
       <c r="AF6" s="12" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="AG6" s="12" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="AH6" s="13" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="AI6" s="40"/>
       <c r="AJ6" s="12"/>
       <c r="AK6" s="41" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AL6" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="AM6" s="12"/>
       <c r="AN6" s="12"/>
       <c r="AO6" s="13" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="AP6" s="13" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="AQ6" s="12"/>
       <c r="AR6" s="12"/>
@@ -2506,28 +2518,28 @@
     </row>
     <row r="7" ht="28.5" customHeight="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B7" s="34">
         <v>46038.47222222222</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>63</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G7" s="33" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="I7" s="12" t="s">
         <v>68</v>
@@ -2536,7 +2548,7 @@
         <v>69</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="L7" s="12" t="s">
         <v>71</v>
@@ -2551,16 +2563,16 @@
         <v>73</v>
       </c>
       <c r="P7" s="12" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="Q7" s="36">
         <v>36237</v>
       </c>
       <c r="R7" s="12" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="S7" s="12" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="T7" s="37">
         <v>58</v>
@@ -2569,16 +2581,16 @@
         <v>46044</v>
       </c>
       <c r="V7" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W7" s="47">
         <v>46164</v>
       </c>
       <c r="X7" s="12" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="Y7" s="33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Z7" s="33">
         <v>30</v>
@@ -2589,43 +2601,43 @@
       <c r="AD7" s="12"/>
       <c r="AE7" s="12"/>
       <c r="AF7" s="12" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="AG7" s="12" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="AH7" s="13" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="AI7" s="40"/>
       <c r="AJ7" s="12"/>
       <c r="AK7" s="41" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="AL7" s="13" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="AM7" s="12"/>
       <c r="AN7" s="12"/>
       <c r="AO7" s="13" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="AP7" s="13" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="AQ7" s="13" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="AR7" s="12"/>
       <c r="AS7" s="12"/>
       <c r="AT7" s="12"/>
       <c r="AU7" s="12"/>
       <c r="AV7" s="13" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="AW7" s="12"/>
       <c r="AX7" s="12" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="AY7" s="12"/>
       <c r="AZ7" s="12"/>
@@ -2646,28 +2658,28 @@
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B8" s="34">
         <v>46040.631944444445</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>63</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="F8" s="12" t="s">
         <v>65</v>
       </c>
       <c r="G8" s="33" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I8" s="12" t="s">
         <v>68</v>
@@ -2676,13 +2688,13 @@
         <v>69</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="L8" s="12" t="s">
         <v>71</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="N8" s="35">
         <v>93</v>
@@ -2691,16 +2703,16 @@
         <v>73</v>
       </c>
       <c r="P8" s="12" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="Q8" s="36">
         <v>35276</v>
       </c>
       <c r="R8" s="12" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="S8" s="12" t="s">
-        <v>73</v>
+        <v>95</v>
       </c>
       <c r="T8" s="37">
         <v>85</v>
@@ -2709,16 +2721,16 @@
         <v>46047</v>
       </c>
       <c r="V8" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W8" s="12">
         <v>46228</v>
       </c>
       <c r="X8" s="12" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="Y8" s="12" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="Z8" s="33">
         <v>30</v>
@@ -2729,23 +2741,23 @@
       <c r="AD8" s="12"/>
       <c r="AE8" s="12"/>
       <c r="AF8" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="AG8" s="12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="AH8" s="13" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="AI8" s="40"/>
       <c r="AJ8" s="33">
         <v>34</v>
       </c>
       <c r="AK8" s="41" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="AL8" s="12" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="AM8" s="12"/>
       <c r="AN8" s="12"/>
@@ -2754,7 +2766,7 @@
       <c r="AQ8" s="12"/>
       <c r="AR8" s="12"/>
       <c r="AS8" s="13" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="AT8" s="12"/>
       <c r="AU8" s="12"/>
@@ -2762,7 +2774,7 @@
       <c r="AW8" s="12"/>
       <c r="AX8" s="12"/>
       <c r="AY8" s="13" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="AZ8" s="12"/>
       <c r="BA8" s="12"/>
@@ -2782,7 +2794,7 @@
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B9" s="34">
         <v>46041.41666666667</v>
@@ -2794,16 +2806,16 @@
         <v>63</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G9" s="33" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I9" s="12" t="s">
         <v>68</v>
@@ -2812,13 +2824,13 @@
         <v>69</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="L9" s="12" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="N9" s="35">
         <v>150</v>
@@ -2827,16 +2839,16 @@
         <v>73</v>
       </c>
       <c r="P9" s="12" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="Q9" s="36">
         <v>37239</v>
       </c>
       <c r="R9" s="12" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="S9" s="12" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="T9" s="37">
         <v>140</v>
@@ -2845,16 +2857,16 @@
         <v>46048</v>
       </c>
       <c r="V9" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W9" s="38">
         <v>46321</v>
       </c>
       <c r="X9" s="12" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="Y9" s="33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Z9" s="33">
         <v>30</v>
@@ -2865,64 +2877,64 @@
       <c r="AD9" s="12"/>
       <c r="AE9" s="12"/>
       <c r="AF9" s="12" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="AG9" s="12" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="AH9" s="13" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="AI9" s="40"/>
       <c r="AJ9" s="33">
         <v>28</v>
       </c>
       <c r="AK9" s="41" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="AL9" s="13" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="AM9" s="12"/>
       <c r="AN9" s="12"/>
       <c r="AO9" s="13" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="AP9" s="13" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="AQ9" s="13" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="AR9" s="12"/>
       <c r="AS9" s="13" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AT9" s="12"/>
       <c r="AU9" s="12"/>
       <c r="AV9" s="13" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="AW9" s="13" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="AX9" s="13" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="AY9" s="13" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="AZ9" s="13" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BA9" s="13" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="BB9" s="12" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="BC9" s="13" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="BD9" s="12"/>
       <c r="BE9" s="12"/>
@@ -2938,28 +2950,28 @@
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B10" s="34">
         <v>46042.72916666667</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D10" s="12" t="s">
         <v>63</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F10" s="12" t="s">
         <v>65</v>
       </c>
       <c r="G10" s="33" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="I10" s="12" t="s">
         <v>68</v>
@@ -2968,13 +2980,13 @@
         <v>69</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="N10" s="35">
         <v>30</v>
@@ -2983,16 +2995,16 @@
         <v>73</v>
       </c>
       <c r="P10" s="12" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="Q10" s="36">
         <v>33856</v>
       </c>
       <c r="R10" s="12" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="S10" s="12" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="T10" s="37">
         <v>25</v>
@@ -3001,16 +3013,16 @@
         <v>46050</v>
       </c>
       <c r="V10" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W10" s="38">
         <v>46140</v>
       </c>
       <c r="X10" s="12" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="Y10" s="12" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="Z10" s="33">
         <v>30</v>
@@ -3021,32 +3033,32 @@
       <c r="AD10" s="12"/>
       <c r="AE10" s="12"/>
       <c r="AF10" s="12" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="AG10" s="12" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="AH10" s="13" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="AI10" s="40"/>
       <c r="AJ10" s="33">
         <v>6</v>
       </c>
       <c r="AK10" s="41" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="AL10" s="13" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AM10" s="12"/>
       <c r="AN10" s="12"/>
       <c r="AO10" s="13" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AP10" s="12"/>
       <c r="AQ10" s="13" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AR10" s="12"/>
       <c r="AS10" s="12"/>
@@ -3074,28 +3086,28 @@
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B11" s="34">
         <v>46044.59375</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>63</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G11" s="33" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="I11" s="12" t="s">
         <v>68</v>
@@ -3104,7 +3116,7 @@
         <v>69</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="L11" s="12" t="s">
         <v>71</v>
@@ -3119,16 +3131,16 @@
         <v>73</v>
       </c>
       <c r="P11" s="12" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="Q11" s="36">
         <v>35570</v>
       </c>
       <c r="R11" s="12" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="S11" s="12" t="s">
-        <v>73</v>
+        <v>95</v>
       </c>
       <c r="T11" s="37">
         <v>52</v>
@@ -3137,16 +3149,16 @@
         <v>46055</v>
       </c>
       <c r="V11" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W11" s="12">
         <v>46175</v>
       </c>
       <c r="X11" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Y11" s="33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Z11" s="33">
         <v>30</v>
@@ -3157,29 +3169,29 @@
       <c r="AD11" s="12"/>
       <c r="AE11" s="12"/>
       <c r="AF11" s="12" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="AG11" s="12" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="AH11" s="13" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AI11" s="40"/>
       <c r="AJ11" s="12"/>
       <c r="AK11" s="41" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="AL11" s="12" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="AM11" s="12"/>
       <c r="AN11" s="12"/>
       <c r="AO11" s="13" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="AP11" s="13" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="AQ11" s="12"/>
       <c r="AR11" s="12"/>
@@ -3208,7 +3220,7 @@
     </row>
     <row r="12" ht="23.25" customHeight="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B12" s="34">
         <v>46047.569444444445</v>
@@ -3220,16 +3232,16 @@
         <v>63</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>65</v>
       </c>
       <c r="G12" s="33" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="I12" s="12" t="s">
         <v>68</v>
@@ -3238,13 +3250,13 @@
         <v>69</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="L12" s="12" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="N12" s="35">
         <v>120</v>
@@ -3253,16 +3265,16 @@
         <v>73</v>
       </c>
       <c r="P12" s="12" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="Q12" s="36">
         <v>34380</v>
       </c>
       <c r="R12" s="12" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="S12" s="12" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="T12" s="37">
         <v>110</v>
@@ -3271,16 +3283,16 @@
         <v>46058</v>
       </c>
       <c r="V12" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W12" s="38">
         <v>46239</v>
       </c>
       <c r="X12" s="12" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="Y12" s="33" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="Z12" s="33">
         <v>30</v>
@@ -3291,29 +3303,29 @@
       <c r="AD12" s="12"/>
       <c r="AE12" s="12"/>
       <c r="AF12" s="12" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="AG12" s="12" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="AH12" s="13" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="AI12" s="40"/>
       <c r="AJ12" s="12"/>
       <c r="AK12" s="41" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AL12" s="13" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="AM12" s="12"/>
       <c r="AN12" s="12"/>
       <c r="AO12" s="12" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="AP12" s="12" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="AQ12" s="12"/>
       <c r="AR12" s="12"/>
@@ -3342,28 +3354,28 @@
     </row>
     <row r="13" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B13" s="34">
         <v>46050.40972222222</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>63</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G13" s="33" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="I13" s="12" t="s">
         <v>68</v>
@@ -3372,13 +3384,13 @@
         <v>69</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="L13" s="12" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="M13" s="12" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="N13" s="35">
         <v>30</v>
@@ -3387,16 +3399,16 @@
         <v>73</v>
       </c>
       <c r="P13" s="12" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="Q13" s="36">
         <v>36809</v>
       </c>
       <c r="R13" s="12" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="S13" s="12" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="T13" s="37">
         <v>28</v>
@@ -3405,16 +3417,16 @@
         <v>46063</v>
       </c>
       <c r="V13" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W13" s="38">
         <v>46152</v>
       </c>
       <c r="X13" s="12" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="Y13" s="33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Z13" s="33">
         <v>30</v>
@@ -3425,30 +3437,30 @@
       <c r="AD13" s="12"/>
       <c r="AE13" s="12"/>
       <c r="AF13" s="12" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="AG13" s="12" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="AH13" s="13" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="AI13" s="40"/>
       <c r="AJ13" s="12"/>
       <c r="AK13" s="41" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="AL13" s="13" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="AM13" s="12"/>
       <c r="AN13" s="12"/>
       <c r="AO13" s="13" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="AP13" s="12"/>
       <c r="AQ13" s="12" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="AR13" s="12"/>
       <c r="AS13" s="12"/>
@@ -3537,7 +3549,7 @@
   <sheetData>
     <row r="1" spans="1:466" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -3570,7 +3582,7 @@
       <c r="AA1" s="12"/>
       <c r="AB1" s="12"/>
       <c r="AC1" s="52" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="AD1" s="12"/>
       <c r="AE1" s="12"/>
@@ -3609,7 +3621,7 @@
       <c r="BL1" s="12"/>
       <c r="BM1" s="12"/>
       <c r="BN1" s="53" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="BO1" s="54"/>
       <c r="BP1" s="54"/>
@@ -3645,7 +3657,7 @@
       <c r="CT1" s="12"/>
       <c r="CU1" s="12"/>
       <c r="CV1" s="52" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="CW1" s="12"/>
       <c r="CX1" s="12"/>
@@ -4055,7 +4067,7 @@
         <v>9</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>20</v>
+        <v>217</v>
       </c>
       <c r="I2" s="74" t="s">
         <v>21</v>
@@ -4103,37 +4115,37 @@
         <v>35</v>
       </c>
       <c r="X2" s="29" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="Y2" s="29" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="Z2" s="76" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="AA2" s="76" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="AB2" s="76" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="AC2" s="77" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="AD2" s="77" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="AE2" s="77" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="AF2" s="77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="AG2" s="77" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="AH2" s="77" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="AI2" s="78">
         <v>46023</v>
@@ -4229,22 +4241,22 @@
         <v>46053</v>
       </c>
       <c r="BN2" s="79" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="BO2" s="79" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="BP2" s="79" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="BQ2" s="79" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="BR2" s="79" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="BS2" s="79" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="BT2" s="78">
         <v>46054</v>
@@ -4331,22 +4343,22 @@
         <v>46081</v>
       </c>
       <c r="CV2" s="77" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="CW2" s="77" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="CX2" s="77" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="CY2" s="77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="CZ2" s="77" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="DA2" s="77" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="DB2" s="78">
         <v>46082</v>
@@ -4442,22 +4454,22 @@
         <v>46112</v>
       </c>
       <c r="EG2" s="77" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="EH2" s="77" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="EI2" s="77" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="EJ2" s="77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="EK2" s="77" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="EL2" s="77" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="EM2" s="78">
         <v>46113</v>
@@ -4550,22 +4562,22 @@
         <v>46142</v>
       </c>
       <c r="FQ2" s="77" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="FR2" s="77" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="FS2" s="77" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="FT2" s="77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="FU2" s="77" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="FV2" s="77" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="FW2" s="80">
         <v>46143</v>
@@ -4661,22 +4673,22 @@
         <v>46173</v>
       </c>
       <c r="HB2" s="79" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="HC2" s="79" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="HD2" s="79" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="HE2" s="79" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="HF2" s="79" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="HG2" s="79" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="HH2" s="78">
         <v>46174</v>
@@ -4769,22 +4781,22 @@
         <v>46203</v>
       </c>
       <c r="IL2" s="82" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="IM2" s="77" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="IN2" s="77" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="IO2" s="77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="IP2" s="77" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="IQ2" s="83" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="IR2" s="78">
         <v>46204</v>
@@ -4880,22 +4892,22 @@
         <v>46234</v>
       </c>
       <c r="JW2" s="77" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="JX2" s="77" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="JY2" s="77" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="JZ2" s="77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="KA2" s="77" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="KB2" s="77" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="KC2" s="78">
         <v>46235</v>
@@ -4991,22 +5003,22 @@
         <v>46265</v>
       </c>
       <c r="LH2" s="77" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="LI2" s="77" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="LJ2" s="77" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="LK2" s="77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="LL2" s="77" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="LM2" s="77" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="LN2" s="78">
         <v>46266</v>
@@ -5099,22 +5111,22 @@
         <f>MP2+1</f>
       </c>
       <c r="MR2" s="77" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="MS2" s="77" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="MT2" s="77" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="MU2" s="77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="MV2" s="77" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="MW2" s="77" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="MX2" s="78">
         <v>46296</v>
@@ -5210,22 +5222,22 @@
         <f>OA2+1</f>
       </c>
       <c r="OC2" s="77" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="OD2" s="77" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="OE2" s="77" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="OF2" s="77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="OG2" s="77" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="OH2" s="77" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="OI2" s="78">
         <v>46327</v>
@@ -5318,22 +5330,22 @@
         <f>PK2+1</f>
       </c>
       <c r="PM2" s="77" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="PN2" s="77" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="PO2" s="77" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="PP2" s="77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="PQ2" s="77" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="PR2" s="77" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="PS2" s="78">
         <v>46357</v>
@@ -5464,16 +5476,16 @@
         <v>46037</v>
       </c>
       <c r="K3" s="47" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L3" s="91">
         <v>46127</v>
       </c>
       <c r="M3" s="49" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N3" s="64" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O3" s="64">
         <v>30</v>
@@ -5484,13 +5496,13 @@
       <c r="S3" s="49"/>
       <c r="T3" s="49"/>
       <c r="U3" s="49" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="V3" s="49" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="W3" s="92" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="X3" s="89">
         <v>9</v>
@@ -5526,16 +5538,16 @@
         <v>0</v>
       </c>
       <c r="AX3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BA3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BC3" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BE3" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="BN3" s="94">
         <v>0</v>
@@ -5719,13 +5731,13 @@
     </row>
     <row r="4" spans="1:466" x14ac:dyDescent="0.25">
       <c r="A4" s="87" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4" s="87" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C4" s="87" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D4" s="87" t="s">
         <v>68</v>
@@ -5737,7 +5749,7 @@
         <v>71</v>
       </c>
       <c r="G4" s="87" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H4" s="87" t="s">
         <v>73</v>
@@ -5749,16 +5761,16 @@
         <v>46040</v>
       </c>
       <c r="K4" s="47" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L4" s="91">
         <v>46191</v>
       </c>
       <c r="M4" s="49" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N4" s="64" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O4" s="64">
         <v>30</v>
@@ -5769,13 +5781,13 @@
       <c r="S4" s="49"/>
       <c r="T4" s="49"/>
       <c r="U4" s="49" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="V4" s="49" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="W4" s="92" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="X4" s="102">
         <v>15</v>
@@ -5837,15 +5849,15 @@
       </c>
       <c r="AZ4" s="104"/>
       <c r="BA4" s="104" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BB4" s="104"/>
       <c r="BC4" s="104" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BD4" s="104"/>
       <c r="BE4" s="104" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="BF4" s="104"/>
       <c r="BG4" s="104">
@@ -6043,13 +6055,13 @@
     </row>
     <row r="5" spans="1:466" x14ac:dyDescent="0.25">
       <c r="A5" s="87" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B5" s="87" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C5" s="87" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D5" s="87" t="s">
         <v>68</v>
@@ -6061,7 +6073,7 @@
         <v>71</v>
       </c>
       <c r="G5" s="87" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H5" s="87" t="s">
         <v>73</v>
@@ -6073,16 +6085,16 @@
         <v>46042</v>
       </c>
       <c r="K5" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L5" s="91">
         <v>46162</v>
       </c>
       <c r="M5" s="49" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="N5" s="64" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="O5" s="64">
         <v>30</v>
@@ -6093,13 +6105,13 @@
       <c r="S5" s="49"/>
       <c r="T5" s="49"/>
       <c r="U5" s="49" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="V5" s="49" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="W5" s="92" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="X5" s="89">
         <v>10</v>
@@ -6178,17 +6190,17 @@
       <c r="AZ5" s="104"/>
       <c r="BA5" s="104"/>
       <c r="BB5" s="104" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BC5" s="104"/>
       <c r="BD5" s="104" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BE5" s="104">
         <v>0</v>
       </c>
       <c r="BF5" s="104" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BG5" s="104">
         <v>0</v>
@@ -6475,13 +6487,13 @@
     </row>
     <row r="6" spans="1:466" x14ac:dyDescent="0.25">
       <c r="A6" s="105" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B6" s="105" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C6" s="87" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D6" s="87" t="s">
         <v>68</v>
@@ -6493,7 +6505,7 @@
         <v>71</v>
       </c>
       <c r="G6" s="87" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H6" s="87" t="s">
         <v>73</v>
@@ -6505,16 +6517,16 @@
         <v>46044</v>
       </c>
       <c r="K6" s="47" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L6" s="91">
         <v>46164</v>
       </c>
       <c r="M6" s="49" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="N6" s="64" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O6" s="64">
         <v>30</v>
@@ -6527,13 +6539,13 @@
       <c r="S6" s="49"/>
       <c r="T6" s="49"/>
       <c r="U6" s="49" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="V6" s="49" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="W6" s="92" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="X6" s="89">
         <v>2</v>
@@ -6595,12 +6607,12 @@
       <c r="BC6" s="104"/>
       <c r="BD6" s="104"/>
       <c r="BE6" s="104" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BF6" s="104"/>
       <c r="BG6" s="104"/>
       <c r="BH6" s="104" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BI6" s="104"/>
       <c r="BJ6" s="104"/>
@@ -7057,13 +7069,13 @@
     </row>
     <row r="7" spans="1:466" x14ac:dyDescent="0.25">
       <c r="A7" s="87" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B7" s="87" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C7" s="87" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D7" s="87" t="s">
         <v>68</v>
@@ -7075,7 +7087,7 @@
         <v>71</v>
       </c>
       <c r="G7" s="87" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="H7" s="87" t="s">
         <v>73</v>
@@ -7087,16 +7099,16 @@
         <v>46047</v>
       </c>
       <c r="K7" s="91" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L7" s="91">
         <v>46228</v>
       </c>
       <c r="M7" s="49" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="N7" s="64" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="O7" s="64">
         <v>30</v>
@@ -7107,13 +7119,13 @@
       <c r="S7" s="49"/>
       <c r="T7" s="49"/>
       <c r="U7" s="49" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="V7" s="49" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="W7" s="92" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="X7" s="104">
         <v>8</v>
@@ -7149,10 +7161,10 @@
         <v>0</v>
       </c>
       <c r="BI7" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BK7" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BN7" s="94">
         <v>0</v>
@@ -7339,13 +7351,13 @@
     </row>
     <row r="8" spans="1:466" x14ac:dyDescent="0.25">
       <c r="A8" s="87" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B8" s="87" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C8" s="87" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D8" s="87" t="s">
         <v>68</v>
@@ -7354,10 +7366,10 @@
         <v>150</v>
       </c>
       <c r="F8" s="87" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="G8" s="87" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="H8" s="87" t="s">
         <v>73</v>
@@ -7369,16 +7381,16 @@
         <v>46048</v>
       </c>
       <c r="K8" s="111" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L8" s="91">
         <v>46321</v>
       </c>
       <c r="M8" s="49" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="N8" s="64" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O8" s="64">
         <v>30</v>
@@ -7389,13 +7401,13 @@
       <c r="S8" s="49"/>
       <c r="T8" s="49"/>
       <c r="U8" s="49" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="V8" s="49" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="W8" s="112" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="X8" s="104">
         <v>10</v>
@@ -7431,10 +7443,10 @@
         <v>0</v>
       </c>
       <c r="BJ8" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BL8" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BN8" s="94">
         <v>0</v>
@@ -8060,13 +8072,13 @@
     </row>
     <row r="9" spans="1:466" x14ac:dyDescent="0.25">
       <c r="A9" s="87" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B9" s="87" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C9" s="87" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D9" s="87" t="s">
         <v>68</v>
@@ -8075,10 +8087,10 @@
         <v>30</v>
       </c>
       <c r="F9" s="87" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="G9" s="87" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="H9" s="87" t="s">
         <v>73</v>
@@ -8090,16 +8102,16 @@
         <v>46050</v>
       </c>
       <c r="K9" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L9" s="91">
         <v>46140</v>
       </c>
       <c r="M9" s="49" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="N9" s="64" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="O9" s="64">
         <v>30</v>
@@ -8110,13 +8122,13 @@
       <c r="S9" s="49"/>
       <c r="T9" s="49"/>
       <c r="U9" s="49" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="V9" s="49" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="W9" s="92" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="X9" s="104">
         <v>5</v>
@@ -8152,10 +8164,10 @@
         <v>0</v>
       </c>
       <c r="BK9" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BM9" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BN9" s="94">
         <v>0</v>
@@ -8357,13 +8369,13 @@
     </row>
     <row r="10" spans="1:466" x14ac:dyDescent="0.25">
       <c r="A10" s="87" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B10" s="87" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C10" s="87" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D10" s="87" t="s">
         <v>68</v>
@@ -8375,7 +8387,7 @@
         <v>71</v>
       </c>
       <c r="G10" s="87" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H10" s="87" t="s">
         <v>73</v>
@@ -8387,16 +8399,16 @@
         <v>46055</v>
       </c>
       <c r="K10" s="49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L10" s="91">
         <v>46175</v>
       </c>
       <c r="M10" s="49" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N10" s="64" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O10" s="64">
         <v>30</v>
@@ -8407,13 +8419,13 @@
       <c r="S10" s="49"/>
       <c r="T10" s="49"/>
       <c r="U10" s="49" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="V10" s="49" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="W10" s="92" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="X10" s="104">
         <v>8</v>
@@ -8467,10 +8479,10 @@
         <v>0</v>
       </c>
       <c r="BU10" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BW10" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="CV10" s="95">
         <v>0</v>
@@ -8631,7 +8643,7 @@
         <v>0</v>
       </c>
       <c r="LP10" s="115" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="LQ10" s="115">
         <v>2</v>
@@ -8645,13 +8657,13 @@
     </row>
     <row r="11" spans="1:466" x14ac:dyDescent="0.25">
       <c r="A11" s="87" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B11" s="87" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C11" s="87" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D11" s="87" t="s">
         <v>68</v>
@@ -8660,10 +8672,10 @@
         <v>120</v>
       </c>
       <c r="F11" s="87" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="G11" s="87" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="H11" s="87" t="s">
         <v>73</v>
@@ -8675,16 +8687,16 @@
         <v>46058</v>
       </c>
       <c r="K11" s="91" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L11" s="91">
         <v>46239</v>
       </c>
       <c r="M11" s="49" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="N11" s="64" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="O11" s="64">
         <v>30</v>
@@ -8695,13 +8707,13 @@
       <c r="S11" s="49"/>
       <c r="T11" s="49"/>
       <c r="U11" s="49" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="V11" s="49" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="W11" s="92" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="X11" s="104">
         <v>10</v>
@@ -8755,10 +8767,10 @@
         <v>0</v>
       </c>
       <c r="BX11" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="BZ11" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="CV11" s="95">
         <v>0</v>
@@ -8924,13 +8936,13 @@
     </row>
     <row r="12" spans="1:466" x14ac:dyDescent="0.25">
       <c r="A12" s="87" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B12" s="87" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C12" s="87" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D12" s="87" t="s">
         <v>68</v>
@@ -8939,10 +8951,10 @@
         <v>30</v>
       </c>
       <c r="F12" s="87" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="G12" s="87" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="H12" s="87" t="s">
         <v>73</v>
@@ -8954,16 +8966,16 @@
         <v>46063</v>
       </c>
       <c r="K12" s="91" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L12" s="91">
         <v>46152</v>
       </c>
       <c r="M12" s="49" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="N12" s="64" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O12" s="64">
         <v>30</v>
@@ -8974,13 +8986,13 @@
       <c r="S12" s="49"/>
       <c r="T12" s="49"/>
       <c r="U12" s="49" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="V12" s="49" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="W12" s="92" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="X12" s="103">
         <v>2</v>
@@ -9034,10 +9046,10 @@
         <v>0</v>
       </c>
       <c r="CD12" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="CF12" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="CV12" s="95">
         <v>0</v>

</xml_diff>